<commit_message>
new changes for MIS
</commit_message>
<xml_diff>
--- a/agreement.xlsx
+++ b/agreement.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\shyam\Documents\Dev\sol-emp-accomodation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D49E5743-67CE-4459-A929-E911F96B5673}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90CC27C5-E17D-4146-BD76-DC70A86F92C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{500B3CF0-1DE7-4087-874E-66A7CEAD6D1B}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{500B3CF0-1DE7-4087-874E-66A7CEAD6D1B}"/>
   </bookViews>
   <sheets>
     <sheet name="residence_master" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7044" uniqueCount="2140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7046" uniqueCount="2142">
   <si>
     <t>L Saraswathi (w/o Ramesh D)</t>
   </si>
@@ -6462,6 +6462,12 @@
   </si>
   <si>
     <t>INACTIVE</t>
+  </si>
+  <si>
+    <t>agreement_amount_received</t>
+  </si>
+  <si>
+    <t>agreement_set_to_vacate</t>
   </si>
 </sst>
 </file>
@@ -10029,7 +10035,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3CB4CCAD-08D6-4AED-9516-35C0E7D84C9E}">
-  <dimension ref="A1:H83"/>
+  <dimension ref="A1:J83"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15.88671875" style="3" customWidth="1"/>
@@ -10039,10 +10045,12 @@
     <col min="5" max="5" width="22" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="26.33203125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="30.88671875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="21.44140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.21875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="26.33203125" customWidth="1"/>
+    <col min="10" max="10" width="23.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>2125</v>
       </c>
@@ -10067,8 +10075,14 @@
       <c r="H1" s="1" t="s">
         <v>326</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I1" s="1" t="s">
+        <v>2140</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>2141</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>328</v>
       </c>
@@ -10093,8 +10107,10 @@
       <c r="H2" s="9" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I2" s="9"/>
+      <c r="J2" s="9"/>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>329</v>
       </c>
@@ -10119,8 +10135,10 @@
       <c r="H3" s="9" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I3" s="9"/>
+      <c r="J3" s="9"/>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
         <v>330</v>
       </c>
@@ -10145,8 +10163,10 @@
       <c r="H4" s="9" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I4" s="9"/>
+      <c r="J4" s="9"/>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
         <v>331</v>
       </c>
@@ -10171,8 +10191,10 @@
       <c r="H5" s="9" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I5" s="9"/>
+      <c r="J5" s="9"/>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
         <v>332</v>
       </c>
@@ -10197,8 +10219,10 @@
       <c r="H6" s="9" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I6" s="9"/>
+      <c r="J6" s="9"/>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
         <v>333</v>
       </c>
@@ -10223,8 +10247,10 @@
       <c r="H7" s="9" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I7" s="9"/>
+      <c r="J7" s="9"/>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
         <v>334</v>
       </c>
@@ -10249,8 +10275,10 @@
       <c r="H8" s="9" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I8" s="9"/>
+      <c r="J8" s="9"/>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
         <v>335</v>
       </c>
@@ -10275,8 +10303,10 @@
       <c r="H9" s="9" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I9" s="9"/>
+      <c r="J9" s="9"/>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
         <v>336</v>
       </c>
@@ -10301,8 +10331,10 @@
       <c r="H10" s="9" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I10" s="9"/>
+      <c r="J10" s="9"/>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
         <v>337</v>
       </c>
@@ -10327,8 +10359,10 @@
       <c r="H11" s="9" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I11" s="9"/>
+      <c r="J11" s="9"/>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
         <v>338</v>
       </c>
@@ -10353,8 +10387,10 @@
       <c r="H12" s="9" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I12" s="9"/>
+      <c r="J12" s="9"/>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
         <v>339</v>
       </c>
@@ -10379,8 +10415,10 @@
       <c r="H13" s="9" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I13" s="9"/>
+      <c r="J13" s="9"/>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
         <v>340</v>
       </c>
@@ -10405,8 +10443,10 @@
       <c r="H14" s="9" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I14" s="9"/>
+      <c r="J14" s="9"/>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A15" s="4" t="s">
         <v>341</v>
       </c>
@@ -10431,8 +10471,10 @@
       <c r="H15" s="9" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I15" s="9"/>
+      <c r="J15" s="9"/>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A16" s="4" t="s">
         <v>342</v>
       </c>
@@ -10457,8 +10499,10 @@
       <c r="H16" s="9" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I16" s="9"/>
+      <c r="J16" s="9"/>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A17" s="4" t="s">
         <v>343</v>
       </c>
@@ -10483,8 +10527,10 @@
       <c r="H17" s="9" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I17" s="9"/>
+      <c r="J17" s="9"/>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
         <v>344</v>
       </c>
@@ -10509,8 +10555,10 @@
       <c r="H18" s="9" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I18" s="9"/>
+      <c r="J18" s="9"/>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
         <v>345</v>
       </c>
@@ -10535,8 +10583,10 @@
       <c r="H19" s="9" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I19" s="9"/>
+      <c r="J19" s="9"/>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A20" s="4" t="s">
         <v>346</v>
       </c>
@@ -10561,8 +10611,10 @@
       <c r="H20" s="9" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I20" s="9"/>
+      <c r="J20" s="9"/>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A21" s="4" t="s">
         <v>347</v>
       </c>
@@ -10587,8 +10639,10 @@
       <c r="H21" s="9" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I21" s="9"/>
+      <c r="J21" s="9"/>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A22" s="4" t="s">
         <v>348</v>
       </c>
@@ -10613,8 +10667,10 @@
       <c r="H22" s="9" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I22" s="9"/>
+      <c r="J22" s="9"/>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A23" s="4" t="s">
         <v>349</v>
       </c>
@@ -10639,8 +10695,10 @@
       <c r="H23" s="9" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I23" s="9"/>
+      <c r="J23" s="9"/>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A24" s="4" t="s">
         <v>350</v>
       </c>
@@ -10665,8 +10723,10 @@
       <c r="H24" s="9" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I24" s="9"/>
+      <c r="J24" s="9"/>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A25" s="4" t="s">
         <v>351</v>
       </c>
@@ -10691,8 +10751,10 @@
       <c r="H25" s="9" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I25" s="9"/>
+      <c r="J25" s="9"/>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A26" s="4" t="s">
         <v>352</v>
       </c>
@@ -10717,8 +10779,10 @@
       <c r="H26" s="9" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I26" s="9"/>
+      <c r="J26" s="9"/>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A27" s="4" t="s">
         <v>353</v>
       </c>
@@ -10743,8 +10807,10 @@
       <c r="H27" s="9" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I27" s="9"/>
+      <c r="J27" s="9"/>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A28" s="4" t="s">
         <v>354</v>
       </c>
@@ -10769,8 +10835,10 @@
       <c r="H28" s="9" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I28" s="9"/>
+      <c r="J28" s="9"/>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A29" s="4" t="s">
         <v>355</v>
       </c>
@@ -10795,8 +10863,10 @@
       <c r="H29" s="9" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I29" s="9"/>
+      <c r="J29" s="9"/>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A30" s="4" t="s">
         <v>356</v>
       </c>
@@ -10821,8 +10891,10 @@
       <c r="H30" s="9" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I30" s="9"/>
+      <c r="J30" s="9"/>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A31" s="4" t="s">
         <v>357</v>
       </c>
@@ -10847,8 +10919,10 @@
       <c r="H31" s="9" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I31" s="9"/>
+      <c r="J31" s="9"/>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A32" s="4" t="s">
         <v>358</v>
       </c>
@@ -10873,8 +10947,10 @@
       <c r="H32" s="9" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I32" s="9"/>
+      <c r="J32" s="9"/>
+    </row>
+    <row r="33" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A33" s="4" t="s">
         <v>359</v>
       </c>
@@ -10899,8 +10975,10 @@
       <c r="H33" s="9" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I33" s="9"/>
+      <c r="J33" s="9"/>
+    </row>
+    <row r="34" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A34" s="4" t="s">
         <v>360</v>
       </c>
@@ -10925,8 +11003,10 @@
       <c r="H34" s="9" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I34" s="9"/>
+      <c r="J34" s="9"/>
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A35" s="4" t="s">
         <v>361</v>
       </c>
@@ -10951,8 +11031,10 @@
       <c r="H35" s="9" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I35" s="9"/>
+      <c r="J35" s="9"/>
+    </row>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A36" s="4" t="s">
         <v>362</v>
       </c>
@@ -10977,8 +11059,10 @@
       <c r="H36" s="9" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I36" s="9"/>
+      <c r="J36" s="9"/>
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A37" s="4" t="s">
         <v>363</v>
       </c>
@@ -11003,8 +11087,10 @@
       <c r="H37" s="9" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I37" s="9"/>
+      <c r="J37" s="9"/>
+    </row>
+    <row r="38" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A38" s="4" t="s">
         <v>364</v>
       </c>
@@ -11029,8 +11115,10 @@
       <c r="H38" s="9" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I38" s="9"/>
+      <c r="J38" s="9"/>
+    </row>
+    <row r="39" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A39" s="4" t="s">
         <v>365</v>
       </c>
@@ -11055,8 +11143,10 @@
       <c r="H39" s="9" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I39" s="9"/>
+      <c r="J39" s="9"/>
+    </row>
+    <row r="40" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A40" s="4" t="s">
         <v>366</v>
       </c>
@@ -11081,8 +11171,10 @@
       <c r="H40" s="9" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I40" s="9"/>
+      <c r="J40" s="9"/>
+    </row>
+    <row r="41" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A41" s="4" t="s">
         <v>367</v>
       </c>
@@ -11107,8 +11199,10 @@
       <c r="H41" s="9" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I41" s="9"/>
+      <c r="J41" s="9"/>
+    </row>
+    <row r="42" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A42" s="4" t="s">
         <v>368</v>
       </c>
@@ -11133,8 +11227,10 @@
       <c r="H42" s="9" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I42" s="9"/>
+      <c r="J42" s="9"/>
+    </row>
+    <row r="43" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A43" s="4" t="s">
         <v>369</v>
       </c>
@@ -11159,8 +11255,10 @@
       <c r="H43" s="9" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I43" s="9"/>
+      <c r="J43" s="9"/>
+    </row>
+    <row r="44" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A44" s="4" t="s">
         <v>370</v>
       </c>
@@ -11185,8 +11283,10 @@
       <c r="H44" s="9" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I44" s="9"/>
+      <c r="J44" s="9"/>
+    </row>
+    <row r="45" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A45" s="4" t="s">
         <v>371</v>
       </c>
@@ -11211,8 +11311,10 @@
       <c r="H45" s="9" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I45" s="9"/>
+      <c r="J45" s="9"/>
+    </row>
+    <row r="46" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A46" s="4" t="s">
         <v>372</v>
       </c>
@@ -11237,8 +11339,10 @@
       <c r="H46" s="9" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I46" s="9"/>
+      <c r="J46" s="9"/>
+    </row>
+    <row r="47" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A47" s="4" t="s">
         <v>373</v>
       </c>
@@ -11263,8 +11367,10 @@
       <c r="H47" s="9" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I47" s="9"/>
+      <c r="J47" s="9"/>
+    </row>
+    <row r="48" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A48" s="4" t="s">
         <v>374</v>
       </c>
@@ -11289,8 +11395,10 @@
       <c r="H48" s="9" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I48" s="9"/>
+      <c r="J48" s="9"/>
+    </row>
+    <row r="49" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A49" s="4" t="s">
         <v>375</v>
       </c>
@@ -11315,8 +11423,10 @@
       <c r="H49" s="9" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I49" s="9"/>
+      <c r="J49" s="9"/>
+    </row>
+    <row r="50" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A50" s="4" t="s">
         <v>376</v>
       </c>
@@ -11341,8 +11451,10 @@
       <c r="H50" s="9" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I50" s="9"/>
+      <c r="J50" s="9"/>
+    </row>
+    <row r="51" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A51" s="4" t="s">
         <v>377</v>
       </c>
@@ -11367,8 +11479,10 @@
       <c r="H51" s="9" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I51" s="9"/>
+      <c r="J51" s="9"/>
+    </row>
+    <row r="52" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A52" s="4" t="s">
         <v>378</v>
       </c>
@@ -11393,8 +11507,10 @@
       <c r="H52" s="9" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I52" s="9"/>
+      <c r="J52" s="9"/>
+    </row>
+    <row r="53" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A53" s="4" t="s">
         <v>379</v>
       </c>
@@ -11419,8 +11535,10 @@
       <c r="H53" s="9" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I53" s="9"/>
+      <c r="J53" s="9"/>
+    </row>
+    <row r="54" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A54" s="4" t="s">
         <v>380</v>
       </c>
@@ -11445,8 +11563,10 @@
       <c r="H54" s="9" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I54" s="9"/>
+      <c r="J54" s="9"/>
+    </row>
+    <row r="55" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A55" s="4" t="s">
         <v>381</v>
       </c>
@@ -11471,8 +11591,10 @@
       <c r="H55" s="9" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I55" s="9"/>
+      <c r="J55" s="9"/>
+    </row>
+    <row r="56" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A56" s="4" t="s">
         <v>382</v>
       </c>
@@ -11497,8 +11619,10 @@
       <c r="H56" s="9" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="57" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I56" s="9"/>
+      <c r="J56" s="9"/>
+    </row>
+    <row r="57" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A57" s="4" t="s">
         <v>383</v>
       </c>
@@ -11523,8 +11647,10 @@
       <c r="H57" s="9" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I57" s="9"/>
+      <c r="J57" s="9"/>
+    </row>
+    <row r="58" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A58" s="4" t="s">
         <v>384</v>
       </c>
@@ -11549,8 +11675,10 @@
       <c r="H58" s="9" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I58" s="9"/>
+      <c r="J58" s="9"/>
+    </row>
+    <row r="59" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A59" s="4" t="s">
         <v>385</v>
       </c>
@@ -11575,8 +11703,10 @@
       <c r="H59" s="9" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I59" s="9"/>
+      <c r="J59" s="9"/>
+    </row>
+    <row r="60" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A60" s="4" t="s">
         <v>386</v>
       </c>
@@ -11601,8 +11731,10 @@
       <c r="H60" s="9" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="61" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I60" s="9"/>
+      <c r="J60" s="9"/>
+    </row>
+    <row r="61" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A61" s="4" t="s">
         <v>387</v>
       </c>
@@ -11627,8 +11759,10 @@
       <c r="H61" s="9" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I61" s="9"/>
+      <c r="J61" s="9"/>
+    </row>
+    <row r="62" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A62" s="4" t="s">
         <v>388</v>
       </c>
@@ -11653,8 +11787,10 @@
       <c r="H62" s="9" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="63" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I62" s="9"/>
+      <c r="J62" s="9"/>
+    </row>
+    <row r="63" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A63" s="4" t="s">
         <v>389</v>
       </c>
@@ -11679,8 +11815,10 @@
       <c r="H63" s="9" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="64" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I63" s="9"/>
+      <c r="J63" s="9"/>
+    </row>
+    <row r="64" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A64" s="4" t="s">
         <v>390</v>
       </c>
@@ -11705,8 +11843,10 @@
       <c r="H64" s="9" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="65" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I64" s="9"/>
+      <c r="J64" s="9"/>
+    </row>
+    <row r="65" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A65" s="4" t="s">
         <v>391</v>
       </c>
@@ -11731,8 +11871,10 @@
       <c r="H65" s="9" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="66" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I65" s="9"/>
+      <c r="J65" s="9"/>
+    </row>
+    <row r="66" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A66" s="4" t="s">
         <v>392</v>
       </c>
@@ -11757,8 +11899,10 @@
       <c r="H66" s="9" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="67" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I66" s="9"/>
+      <c r="J66" s="9"/>
+    </row>
+    <row r="67" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A67" s="4" t="s">
         <v>393</v>
       </c>
@@ -11783,8 +11927,10 @@
       <c r="H67" s="9" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="68" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I67" s="9"/>
+      <c r="J67" s="9"/>
+    </row>
+    <row r="68" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A68" s="4" t="s">
         <v>394</v>
       </c>
@@ -11809,8 +11955,10 @@
       <c r="H68" s="9" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="69" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I68" s="9"/>
+      <c r="J68" s="9"/>
+    </row>
+    <row r="69" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A69" s="4" t="s">
         <v>395</v>
       </c>
@@ -11835,8 +11983,10 @@
       <c r="H69" s="9" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="70" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I69" s="9"/>
+      <c r="J69" s="9"/>
+    </row>
+    <row r="70" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A70" s="4" t="s">
         <v>396</v>
       </c>
@@ -11861,8 +12011,10 @@
       <c r="H70" s="9" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="71" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I70" s="9"/>
+      <c r="J70" s="9"/>
+    </row>
+    <row r="71" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A71" s="4" t="s">
         <v>397</v>
       </c>
@@ -11887,8 +12039,10 @@
       <c r="H71" s="9" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="72" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I71" s="9"/>
+      <c r="J71" s="9"/>
+    </row>
+    <row r="72" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A72" s="4" t="s">
         <v>398</v>
       </c>
@@ -11913,8 +12067,10 @@
       <c r="H72" s="9" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="73" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I72" s="9"/>
+      <c r="J72" s="9"/>
+    </row>
+    <row r="73" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A73" s="4" t="s">
         <v>399</v>
       </c>
@@ -11939,8 +12095,10 @@
       <c r="H73" s="9" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="74" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I73" s="9"/>
+      <c r="J73" s="9"/>
+    </row>
+    <row r="74" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A74" s="4" t="s">
         <v>400</v>
       </c>
@@ -11965,8 +12123,10 @@
       <c r="H74" s="9" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="75" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I74" s="9"/>
+      <c r="J74" s="9"/>
+    </row>
+    <row r="75" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A75" s="4" t="s">
         <v>401</v>
       </c>
@@ -11991,8 +12151,10 @@
       <c r="H75" s="9" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="76" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I75" s="9"/>
+      <c r="J75" s="9"/>
+    </row>
+    <row r="76" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A76" s="4" t="s">
         <v>402</v>
       </c>
@@ -12017,8 +12179,10 @@
       <c r="H76" s="9" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="77" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I76" s="9"/>
+      <c r="J76" s="9"/>
+    </row>
+    <row r="77" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A77" s="4" t="s">
         <v>403</v>
       </c>
@@ -12043,8 +12207,10 @@
       <c r="H77" s="9" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="78" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I77" s="9"/>
+      <c r="J77" s="9"/>
+    </row>
+    <row r="78" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A78" s="4" t="s">
         <v>404</v>
       </c>
@@ -12069,8 +12235,10 @@
       <c r="H78" s="9" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="79" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I78" s="9"/>
+      <c r="J78" s="9"/>
+    </row>
+    <row r="79" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A79" s="4" t="s">
         <v>405</v>
       </c>
@@ -12095,8 +12263,10 @@
       <c r="H79" s="9" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="80" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I79" s="9"/>
+      <c r="J79" s="9"/>
+    </row>
+    <row r="80" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A80" s="4" t="s">
         <v>406</v>
       </c>
@@ -12121,8 +12291,10 @@
       <c r="H80" s="9" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="81" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I80" s="9"/>
+      <c r="J80" s="9"/>
+    </row>
+    <row r="81" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A81" s="4" t="s">
         <v>407</v>
       </c>
@@ -12147,8 +12319,10 @@
       <c r="H81" s="9" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="82" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I81" s="9"/>
+      <c r="J81" s="9"/>
+    </row>
+    <row r="82" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A82" s="4" t="s">
         <v>408</v>
       </c>
@@ -12173,8 +12347,10 @@
       <c r="H82" s="9" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="83" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I82" s="9"/>
+      <c r="J82" s="9"/>
+    </row>
+    <row r="83" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A83" s="4" t="s">
         <v>409</v>
       </c>
@@ -12199,6 +12375,8 @@
       <c r="H83" s="9" t="s">
         <v>327</v>
       </c>
+      <c r="I83" s="9"/>
+      <c r="J83" s="9"/>
     </row>
   </sheetData>
   <phoneticPr fontId="7" type="noConversion"/>

</xml_diff>